<commit_message>
Limit strategy evaluation template sheets
</commit_message>
<xml_diff>
--- a/assets/template-data-source-strategi-evaluasi.xlsx
+++ b/assets/template-data-source-strategi-evaluasi.xlsx
@@ -2,17 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_Panduan" sheetId="1" r:id="R4f054cae698d4f0f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_Referensi" sheetId="2" r:id="R25ac7abebf724d84"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_Ratifikasi" sheetId="3" r:id="Rb318ee5cc0934525"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_Change_Request" sheetId="4" r:id="R1b345ce01372413e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_Kinerja" sheetId="5" r:id="Rfb9b588b58b246b5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_Penyusunan_Kebijakan" sheetId="6" r:id="R5f69fdbbee534b28"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_Business_Excellence" sheetId="7" r:id="R872ee12fcbb94191"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_Investasi" sheetId="8" r:id="Rdb0e5f9cee3f49c6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_AO_Korporat" sheetId="9" r:id="Rdb50e888a9c04ba6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_AO_Kantor_Pusat" sheetId="10" r:id="R391c3e6ceb2e4986"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_Ringkasan" sheetId="11" r:id="R584265ee3dd34e81"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_Panduan" sheetId="1" r:id="Rb4755d1d39454ace"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_Referensi" sheetId="2" r:id="R54dea560da5a4936"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_Ratifikasi" sheetId="3" r:id="R78aea8ab673a4ad2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_Change_Request" sheetId="4" r:id="R9e1bf52b084844d1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_Kinerja" sheetId="5" r:id="R5803befbcda74ae0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_Penyusunan_Kebijakan" sheetId="6" r:id="Raa791bf4ed3741ab"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_Business_Excellence" sheetId="7" r:id="R80e89810a0db41bf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_Ringkasan" sheetId="8" r:id="Rd33fe9d6ecfa4fc2"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -113,17 +110,6 @@
 </x:table>
 </file>
 
-<file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="10" name="09RingkasanTable" displayName="09RingkasanTable" ref="A1:C8" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:tableColumns count="3">
-    <x:tableColumn id="1" name="Indikator"/>
-    <x:tableColumn id="2" name="Nilai"/>
-    <x:tableColumn id="3" name="Catatan"/>
-  </x:tableColumns>
-  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</x:table>
-</file>
-
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
 <x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="01RatifikasiTable" displayName="01RatifikasiTable" ref="A1:E141" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="5">
@@ -198,33 +184,11 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="06InvestasiTable" displayName="06InvestasiTable" ref="A1:C23" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="09RingkasanTable" displayName="09RingkasanTable" ref="A1:C8" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="3">
-    <x:tableColumn id="1" name="Kode"/>
-    <x:tableColumn id="2" name="Indikator"/>
-    <x:tableColumn id="3" name="Nilai"/>
-  </x:tableColumns>
-  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</x:table>
-</file>
-
-<file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="07AOKorporatTable" displayName="07AOKorporatTable" ref="A1:C9" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:tableColumns count="3">
-    <x:tableColumn id="1" name="Kode"/>
-    <x:tableColumn id="2" name="Indikator"/>
-    <x:tableColumn id="3" name="Nilai"/>
-  </x:tableColumns>
-  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</x:table>
-</file>
-
-<file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="9" name="08AOKantorPusatTable" displayName="08AOKantorPusatTable" ref="A1:C8" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:tableColumns count="3">
-    <x:tableColumn id="1" name="Kode"/>
-    <x:tableColumn id="2" name="Indikator"/>
-    <x:tableColumn id="3" name="Nilai"/>
+    <x:tableColumn id="1" name="Indikator"/>
+    <x:tableColumn id="2" name="Nilai"/>
+    <x:tableColumn id="3" name="Catatan"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -573,101 +537,41 @@
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="9" t="str">
-        <x:v>06_Investasi</x:v>
+        <x:v>09_Ringkasan</x:v>
       </x:c>
       <x:c r="B9" s="9" t="str">
-        <x:v>Parameter menu Investasi</x:v>
+        <x:v>Parameter ringkasan/NKO</x:v>
       </x:c>
       <x:c r="C9" s="9" t="str">
-        <x:v>Jangan ubah Kode, edit hanya kolom Nilai</x:v>
+        <x:v>Nilai NKO wajib 106,84 bila mengikuti PDF Juni 2026</x:v>
       </x:c>
       <x:c r="D9" s="9" t="str">
-        <x:v>Opsional</x:v>
+        <x:v>Ya</x:v>
       </x:c>
       <x:c r="E9" s="9" t="str">
         <x:v>Ya</x:v>
       </x:c>
       <x:c r="F9" s="9" t="str">
-        <x:v>Kode harus tetap</x:v>
+        <x:v>Dipakai untuk mengunci NKO</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="9" t="str">
-        <x:v>07_AO_Korporat</x:v>
+        <x:v>Cara update</x:v>
       </x:c>
       <x:c r="B10" s="9" t="str">
-        <x:v>Parameter AO Korporat</x:v>
+        <x:v>Edit data di file ini / Google Sheets</x:v>
       </x:c>
       <x:c r="C10" s="9" t="str">
-        <x:v>Jangan ubah Kode, edit hanya kolom Nilai</x:v>
+        <x:v>Import ke dashboard atau hubungkan link Google Drive yang sama</x:v>
       </x:c>
       <x:c r="D10" s="9" t="str">
-        <x:v>Opsional</x:v>
+        <x:v>Ya</x:v>
       </x:c>
       <x:c r="E10" s="9" t="str">
         <x:v>Ya</x:v>
       </x:c>
       <x:c r="F10" s="9" t="str">
-        <x:v>Kode harus tetap</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="11">
-      <x:c r="A11" s="9" t="str">
-        <x:v>08_AO_Kantor_Pusat</x:v>
-      </x:c>
-      <x:c r="B11" s="9" t="str">
-        <x:v>Parameter AO Kantor Pusat</x:v>
-      </x:c>
-      <x:c r="C11" s="9" t="str">
-        <x:v>Jangan ubah Kode, edit hanya kolom Nilai</x:v>
-      </x:c>
-      <x:c r="D11" s="9" t="str">
-        <x:v>Opsional</x:v>
-      </x:c>
-      <x:c r="E11" s="9" t="str">
-        <x:v>Ya</x:v>
-      </x:c>
-      <x:c r="F11" s="9" t="str">
-        <x:v>Kode harus tetap</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="12">
-      <x:c r="A12" s="9" t="str">
-        <x:v>09_Ringkasan</x:v>
-      </x:c>
-      <x:c r="B12" s="9" t="str">
-        <x:v>Parameter ringkasan/NKO</x:v>
-      </x:c>
-      <x:c r="C12" s="9" t="str">
-        <x:v>Nilai NKO wajib 106,84 bila mengikuti PDF Juni 2026</x:v>
-      </x:c>
-      <x:c r="D12" s="9" t="str">
-        <x:v>Ya</x:v>
-      </x:c>
-      <x:c r="E12" s="9" t="str">
-        <x:v>Ya</x:v>
-      </x:c>
-      <x:c r="F12" s="9" t="str">
-        <x:v>Dipakai untuk mengunci NKO</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="13">
-      <x:c r="A13" s="9" t="str">
-        <x:v>Cara update</x:v>
-      </x:c>
-      <x:c r="B13" s="9" t="str">
-        <x:v>Edit data di file ini / Google Sheets</x:v>
-      </x:c>
-      <x:c r="C13" s="9" t="str">
-        <x:v>Import ke dashboard atau hubungkan link Google Drive yang sama</x:v>
-      </x:c>
-      <x:c r="D13" s="9" t="str">
-        <x:v>Ya</x:v>
-      </x:c>
-      <x:c r="E13" s="9" t="str">
-        <x:v>Ya</x:v>
-      </x:c>
-      <x:c r="F13" s="9" t="str">
         <x:v>Refresh akan mengikuti data valid terakhir</x:v>
       </x:c>
     </x:row>
@@ -676,216 +580,6 @@
     <x:mergeCell ref="A1:F1"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</x:worksheet>
-</file>
-
-<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:sheetFormatPr defaultRowHeight="15"/>
-  <x:cols>
-    <x:col min="1" max="1" width="26" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="44" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="28" hidden="0" customWidth="1"/>
-  </x:cols>
-  <x:sheetData>
-    <x:row r="1">
-      <x:c r="A1" s="5" t="str">
-        <x:v>Kode</x:v>
-      </x:c>
-      <x:c r="B1" s="5" t="str">
-        <x:v>Indikator</x:v>
-      </x:c>
-      <x:c r="C1" s="5" t="str">
-        <x:v>Nilai</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="2">
-      <x:c r="A2" s="9" t="str">
-        <x:v>period</x:v>
-      </x:c>
-      <x:c r="B2" s="9" t="str">
-        <x:v>Periode</x:v>
-      </x:c>
-      <x:c r="C2" s="9" t="str">
-        <x:v>Juni 2026</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="3">
-      <x:c r="A3" s="9" t="str">
-        <x:v>selectedUnit</x:v>
-      </x:c>
-      <x:c r="B3" s="9" t="str">
-        <x:v>Pilih/Cari Unit</x:v>
-      </x:c>
-      <x:c r="C3" s="9" t="str">
-        <x:v>KPST</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="4">
-      <x:c r="A4" s="9" t="str">
-        <x:v>realization</x:v>
-      </x:c>
-      <x:c r="B4" s="9" t="str">
-        <x:v>Realisasi s.d. Juni 2026</x:v>
-      </x:c>
-      <x:c r="C4" s="9" t="n">
-        <x:v>1389043</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5">
-      <x:c r="A5" s="9" t="str">
-        <x:v>rank</x:v>
-      </x:c>
-      <x:c r="B5" s="9" t="str">
-        <x:v>Peringkat di Holding</x:v>
-      </x:c>
-      <x:c r="C5" s="9" t="str">
-        <x:v>#1 dari 39</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6">
-      <x:c r="A6" s="9" t="str">
-        <x:v>rkap</x:v>
-      </x:c>
-      <x:c r="B6" s="9" t="str">
-        <x:v>RKAP 2026 (AO)</x:v>
-      </x:c>
-      <x:c r="C6" s="9" t="n">
-        <x:v>3647914</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7">
-      <x:c r="A7" s="9" t="str">
-        <x:v>absorption</x:v>
-      </x:c>
-      <x:c r="B7" s="9" t="str">
-        <x:v>Penyerapan thd RKAP 2026</x:v>
-      </x:c>
-      <x:c r="C7" s="9" t="n">
-        <x:v>38</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8">
-      <x:c r="A8" s="9" t="str">
-        <x:v>yoy</x:v>
-      </x:c>
-      <x:c r="B8" s="9" t="str">
-        <x:v>% YoY</x:v>
-      </x:c>
-      <x:c r="C8" s="9" t="n">
-        <x:v>129</x:v>
-      </x:c>
-    </x:row>
-  </x:sheetData>
-  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdb541d0de1d84016"/>
-  </x:tableParts>
-</x:worksheet>
-</file>
-
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
-<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:sheetFormatPr defaultRowHeight="15"/>
-  <x:cols>
-    <x:col min="1" max="1" width="32" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="24" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="58" hidden="0" customWidth="1"/>
-  </x:cols>
-  <x:sheetData>
-    <x:row r="1">
-      <x:c r="A1" s="5" t="str">
-        <x:v>Indikator</x:v>
-      </x:c>
-      <x:c r="B1" s="5" t="str">
-        <x:v>Nilai</x:v>
-      </x:c>
-      <x:c r="C1" s="5" t="str">
-        <x:v>Catatan</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="2">
-      <x:c r="A2" s="9" t="str">
-        <x:v>Nilai NKO</x:v>
-      </x:c>
-      <x:c r="B2" s="9" t="n">
-        <x:v>106.84</x:v>
-      </x:c>
-      <x:c r="C2" s="9" t="str">
-        <x:v>Wajib 106,84 sesuai laporan NKO DIV GA Juni 2026</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="3">
-      <x:c r="A3" s="9" t="str">
-        <x:v>Total Bobot Kinerja</x:v>
-      </x:c>
-      <x:c r="B3" s="9" t="n">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="C3" s="9" t="str">
-        <x:v>Total bobot indikator utama</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="4">
-      <x:c r="A4" s="9" t="str">
-        <x:v>Periode Kinerja</x:v>
-      </x:c>
-      <x:c r="B4" s="9" t="str">
-        <x:v>S.D. Juni 2026</x:v>
-      </x:c>
-      <x:c r="C4" s="9" t="str">
-        <x:v>Ditampilkan pada panel Monitoring Kinerja</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5">
-      <x:c r="A5" s="9" t="str">
-        <x:v>Status Kinerja</x:v>
-      </x:c>
-      <x:c r="B5" s="9" t="str">
-        <x:v>Tercapai</x:v>
-      </x:c>
-      <x:c r="C5" s="9" t="str">
-        <x:v>NKO &gt;= 100</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6">
-      <x:c r="A6" s="9" t="str">
-        <x:v>Total Entitas SH/AP</x:v>
-      </x:c>
-      <x:c r="B6" s="9" t="n">
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="C6" s="9" t="str">
-        <x:v>Dihitung dari sheet ratifikasi</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7">
-      <x:c r="A7" s="9" t="str">
-        <x:v>Total Kebijakan GA</x:v>
-      </x:c>
-      <x:c r="B7" s="9" t="n">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="C7" s="9" t="str">
-        <x:v>Harus 14 kebijakan</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8">
-      <x:c r="A8" s="9" t="str">
-        <x:v>Total Change Request</x:v>
-      </x:c>
-      <x:c r="B8" s="9" t="n">
-        <x:v>9</x:v>
-      </x:c>
-      <x:c r="C8" s="9" t="str">
-        <x:v>Dihitung dari sheet Change Request</x:v>
-      </x:c>
-    </x:row>
-  </x:sheetData>
-  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4ed340955e484e5b"/>
-  </x:tableParts>
 </x:worksheet>
 </file>
 
@@ -1022,7 +716,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf100530dbae34bf3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6a9772622de2458c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3163,7 +2857,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3085d47d1cb04b10"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3e7410fd87ab4cd6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3357,7 +3051,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re06d5db831e340bb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc02bf1138dad451b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3916,7 +3610,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfde9c057f9bb4210"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6a17f4ba8dca4325"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4021,7 +3715,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb1b9c00e932c440e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6eb8f7807c0d4a90"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4111,7 +3805,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R50e2881dfbff4d87"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdaeefcabd3474a28"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4120,384 +3814,103 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="26" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="44" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="72" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="32" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="24" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="58" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
       <x:c r="A1" s="5" t="str">
-        <x:v>Kode</x:v>
+        <x:v>Indikator</x:v>
       </x:c>
       <x:c r="B1" s="5" t="str">
-        <x:v>Indikator</x:v>
+        <x:v>Nilai</x:v>
       </x:c>
       <x:c r="C1" s="5" t="str">
-        <x:v>Nilai</x:v>
+        <x:v>Catatan</x:v>
       </x:c>
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="9" t="str">
-        <x:v>reportDate</x:v>
-      </x:c>
-      <x:c r="B2" s="9" t="str">
-        <x:v>Periode Laporan</x:v>
+        <x:v>Nilai NKO</x:v>
+      </x:c>
+      <x:c r="B2" s="9" t="n">
+        <x:v>106.84</x:v>
       </x:c>
       <x:c r="C2" s="9" t="str">
-        <x:v>Report ANG Investasi - 16 Juli 2026</x:v>
+        <x:v>Wajib 106,84 sesuai laporan NKO DIV GA Juni 2026</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="9" t="str">
-        <x:v>executiveSignal</x:v>
-      </x:c>
-      <x:c r="B3" s="9" t="str">
-        <x:v>Executive Signal</x:v>
+        <x:v>Total Bobot Kinerja</x:v>
+      </x:c>
+      <x:c r="B3" s="9" t="n">
+        <x:v>100</x:v>
       </x:c>
       <x:c r="C3" s="9" t="str">
-        <x:v>AKI terserap 30,43% dari anggaran kas investasi. Fokus utama: evaluasi realisasi Juli, BAPP, rekomposisi AKI, dan percepatan handshake AI 2027.</x:v>
+        <x:v>Total bobot indikator utama</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="9" t="str">
-        <x:v>totalInvestment</x:v>
+        <x:v>Periode Kinerja</x:v>
       </x:c>
       <x:c r="B4" s="9" t="str">
-        <x:v>Total Anggaran Investasi 2026</x:v>
+        <x:v>S.D. Juni 2026</x:v>
       </x:c>
       <x:c r="C4" s="9" t="str">
-        <x:v>10,89 T</x:v>
+        <x:v>Ditampilkan pada panel Monitoring Kinerja</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="9" t="str">
-        <x:v>totalInvestmentNote</x:v>
+        <x:v>Status Kinerja</x:v>
       </x:c>
       <x:c r="B5" s="9" t="str">
-        <x:v>Catatan Total Anggaran Investasi</x:v>
+        <x:v>Tercapai</x:v>
       </x:c>
       <x:c r="C5" s="9" t="str">
-        <x:v>KP 10,64 T + Sarpras Unit 255,31 M</x:v>
+        <x:v>NKO &gt;= 100</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="9" t="str">
-        <x:v>aiRealization</x:v>
-      </x:c>
-      <x:c r="B6" s="9" t="str">
-        <x:v>Realisasi AI s.d. Juni</x:v>
+        <x:v>Total Entitas SH/AP</x:v>
+      </x:c>
+      <x:c r="B6" s="9" t="n">
+        <x:v>10</x:v>
       </x:c>
       <x:c r="C6" s="9" t="str">
-        <x:v>344,27 M</x:v>
+        <x:v>Dihitung dari sheet ratifikasi</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="9" t="str">
-        <x:v>aiRealizationNote</x:v>
-      </x:c>
-      <x:c r="B7" s="9" t="str">
-        <x:v>Catatan Realisasi AI</x:v>
+        <x:v>Total Kebijakan GA</x:v>
+      </x:c>
+      <x:c r="B7" s="9" t="n">
+        <x:v>14</x:v>
       </x:c>
       <x:c r="C7" s="9" t="str">
-        <x:v>3,16% dari total AI terbit</x:v>
+        <x:v>Harus 14 kebijakan</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="9" t="str">
-        <x:v>aiRealizationPct</x:v>
-      </x:c>
-      <x:c r="B8" s="9" t="str">
-        <x:v>Persentase Realisasi AI</x:v>
+        <x:v>Total Change Request</x:v>
+      </x:c>
+      <x:c r="B8" s="9" t="n">
+        <x:v>9</x:v>
       </x:c>
       <x:c r="C8" s="9" t="str">
-        <x:v>3,16%</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9">
-      <x:c r="A9" s="9" t="str">
-        <x:v>akiTotal</x:v>
-      </x:c>
-      <x:c r="B9" s="9" t="str">
-        <x:v>Total AKI 2026</x:v>
-      </x:c>
-      <x:c r="C9" s="9" t="str">
-        <x:v>1,35 T</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="10">
-      <x:c r="A10" s="9" t="str">
-        <x:v>akiTotalNote</x:v>
-      </x:c>
-      <x:c r="B10" s="9" t="str">
-        <x:v>Catatan Total AKI</x:v>
-      </x:c>
-      <x:c r="C10" s="9" t="str">
-        <x:v>KP 1,18 T + Sarpras Unit 178,66 M</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="11">
-      <x:c r="A11" s="9" t="str">
-        <x:v>akiRealization</x:v>
-      </x:c>
-      <x:c r="B11" s="9" t="str">
-        <x:v>Realisasi AKI s.d. Juni</x:v>
-      </x:c>
-      <x:c r="C11" s="9" t="str">
-        <x:v>412,23 M</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="12">
-      <x:c r="A12" s="9" t="str">
-        <x:v>akiRealizationNote</x:v>
-      </x:c>
-      <x:c r="B12" s="9" t="str">
-        <x:v>Catatan Realisasi AKI</x:v>
-      </x:c>
-      <x:c r="C12" s="9" t="str">
-        <x:v>30,43% dari total AKI</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="13">
-      <x:c r="A13" s="9" t="str">
-        <x:v>akiRealizationPct</x:v>
-      </x:c>
-      <x:c r="B13" s="9" t="str">
-        <x:v>Persentase Realisasi AKI</x:v>
-      </x:c>
-      <x:c r="C13" s="9" t="str">
-        <x:v>30,43%</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="14">
-      <x:c r="A14" s="9" t="str">
-        <x:v>akiGaugeNote</x:v>
-      </x:c>
-      <x:c r="B14" s="9" t="str">
-        <x:v>Narasi Gauge AKI</x:v>
-      </x:c>
-      <x:c r="C14" s="9" t="str">
-        <x:v>412,23 M dari total AKI 1.354,51 M sudah terealisasi.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="15">
-      <x:c r="A15" s="9" t="str">
-        <x:v>akiRealizationChip</x:v>
-      </x:c>
-      <x:c r="B15" s="9" t="str">
-        <x:v>Chip Realisasi AKI</x:v>
-      </x:c>
-      <x:c r="C15" s="9" t="str">
-        <x:v>Realisasi 412,23 M</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="16">
-      <x:c r="A16" s="9" t="str">
-        <x:v>akiGapChip</x:v>
-      </x:c>
-      <x:c r="B16" s="9" t="str">
-        <x:v>Chip Sisa AKI</x:v>
-      </x:c>
-      <x:c r="C16" s="9" t="str">
-        <x:v>Sisa 942,28 M</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="17">
-      <x:c r="A17" s="9" t="str">
-        <x:v>akiOfficePct</x:v>
-      </x:c>
-      <x:c r="B17" s="9" t="str">
-        <x:v>Persentase AKI Kantor Pusat</x:v>
-      </x:c>
-      <x:c r="C17" s="9" t="str">
-        <x:v>29,02%</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="18">
-      <x:c r="A18" s="9" t="str">
-        <x:v>akiOfficeNote</x:v>
-      </x:c>
-      <x:c r="B18" s="9" t="str">
-        <x:v>Catatan AKI Kantor Pusat</x:v>
-      </x:c>
-      <x:c r="C18" s="9" t="str">
-        <x:v>341,29 M dari 1.175,85 M</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="19">
-      <x:c r="A19" s="9" t="str">
-        <x:v>akiSarprasPct</x:v>
-      </x:c>
-      <x:c r="B19" s="9" t="str">
-        <x:v>Persentase AKI Sarpras Unit</x:v>
-      </x:c>
-      <x:c r="C19" s="9" t="str">
-        <x:v>39,71%</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="20">
-      <x:c r="A20" s="9" t="str">
-        <x:v>akiSarprasNote</x:v>
-      </x:c>
-      <x:c r="B20" s="9" t="str">
-        <x:v>Catatan AKI Sarpras Unit</x:v>
-      </x:c>
-      <x:c r="C20" s="9" t="str">
-        <x:v>70,94 M dari 178,66 M</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="21">
-      <x:c r="A21" s="9" t="str">
-        <x:v>akiGapPct</x:v>
-      </x:c>
-      <x:c r="B21" s="9" t="str">
-        <x:v>Persentase Gap AKI</x:v>
-      </x:c>
-      <x:c r="C21" s="9" t="str">
-        <x:v>69,57%</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="22">
-      <x:c r="A22" s="9" t="str">
-        <x:v>akiGapNote</x:v>
-      </x:c>
-      <x:c r="B22" s="9" t="str">
-        <x:v>Catatan Gap AKI</x:v>
-      </x:c>
-      <x:c r="C22" s="9" t="str">
-        <x:v>Perlu BAPP &amp; rekomposisi</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="23">
-      <x:c r="A23" s="9" t="str">
-        <x:v>akiInsight</x:v>
-      </x:c>
-      <x:c r="B23" s="9" t="str">
-        <x:v>Insight AKI</x:v>
-      </x:c>
-      <x:c r="C23" s="9" t="str">
-        <x:v>Serapan AKI masih 30,43%. Kantor Pusat menjadi porsi terbesar, sedangkan Sarpras Unit relatif lebih cepat menyerap.</x:v>
+        <x:v>Dihitung dari sheet Change Request</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rae04040117fe4b24"/>
-  </x:tableParts>
-</x:worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:sheetFormatPr defaultRowHeight="15"/>
-  <x:cols>
-    <x:col min="1" max="1" width="26" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="44" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="28" hidden="0" customWidth="1"/>
-  </x:cols>
-  <x:sheetData>
-    <x:row r="1">
-      <x:c r="A1" s="5" t="str">
-        <x:v>Kode</x:v>
-      </x:c>
-      <x:c r="B1" s="5" t="str">
-        <x:v>Indikator</x:v>
-      </x:c>
-      <x:c r="C1" s="5" t="str">
-        <x:v>Nilai</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="2">
-      <x:c r="A2" s="9" t="str">
-        <x:v>period</x:v>
-      </x:c>
-      <x:c r="B2" s="9" t="str">
-        <x:v>Periode</x:v>
-      </x:c>
-      <x:c r="C2" s="9" t="str">
-        <x:v>Mei 2026</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="3">
-      <x:c r="A3" s="9" t="str">
-        <x:v>total</x:v>
-      </x:c>
-      <x:c r="B3" s="9" t="str">
-        <x:v>Realisasi s.d. Mei 2026</x:v>
-      </x:c>
-      <x:c r="C3" s="9" t="n">
-        <x:v>2931185</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="4">
-      <x:c r="A4" s="9" t="str">
-        <x:v>rkap</x:v>
-      </x:c>
-      <x:c r="B4" s="9" t="str">
-        <x:v>RKAP 2026</x:v>
-      </x:c>
-      <x:c r="C4" s="9" t="n">
-        <x:v>8856162</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5">
-      <x:c r="A5" s="9" t="str">
-        <x:v>absorption</x:v>
-      </x:c>
-      <x:c r="B5" s="9" t="str">
-        <x:v>Penyerapan thd RKAP 2026</x:v>
-      </x:c>
-      <x:c r="C5" s="9" t="n">
-        <x:v>33</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6">
-      <x:c r="A6" s="9" t="str">
-        <x:v>targetRate</x:v>
-      </x:c>
-      <x:c r="B6" s="9" t="str">
-        <x:v>Realisasi vs Target s.d. Mei</x:v>
-      </x:c>
-      <x:c r="C6" s="9" t="n">
-        <x:v>82</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7">
-      <x:c r="A7" s="9" t="str">
-        <x:v>projection</x:v>
-      </x:c>
-      <x:c r="B7" s="9" t="str">
-        <x:v>Proyeksi Setahun 2026</x:v>
-      </x:c>
-      <x:c r="C7" s="9" t="n">
-        <x:v>7724829</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8">
-      <x:c r="A8" s="9" t="str">
-        <x:v>projectionRate</x:v>
-      </x:c>
-      <x:c r="B8" s="9" t="str">
-        <x:v>Proyeksi % RKAP</x:v>
-      </x:c>
-      <x:c r="C8" s="9" t="n">
-        <x:v>87</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9">
-      <x:c r="A9" s="9" t="str">
-        <x:v>yoy</x:v>
-      </x:c>
-      <x:c r="B9" s="9" t="str">
-        <x:v>% YoY</x:v>
-      </x:c>
-      <x:c r="C9" s="9" t="n">
-        <x:v>113</x:v>
-      </x:c>
-    </x:row>
-  </x:sheetData>
-  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raa91c7812ebb4b0d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra8a71c537aa54c4d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Merge ratification workbook into strategy template
</commit_message>
<xml_diff>
--- a/assets/template-data-source-strategi-evaluasi.xlsx
+++ b/assets/template-data-source-strategi-evaluasi.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_Panduan" sheetId="1" r:id="Rb4755d1d39454ace"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_Referensi" sheetId="2" r:id="R54dea560da5a4936"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_Ratifikasi" sheetId="3" r:id="R78aea8ab673a4ad2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_Change_Request" sheetId="4" r:id="R9e1bf52b084844d1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_Kinerja" sheetId="5" r:id="R5803befbcda74ae0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_Penyusunan_Kebijakan" sheetId="6" r:id="Raa791bf4ed3741ab"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_Business_Excellence" sheetId="7" r:id="R80e89810a0db41bf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_Ringkasan" sheetId="8" r:id="Rd33fe9d6ecfa4fc2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_Panduan" sheetId="1" r:id="Rfe9dec80608b47e6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_Referensi" sheetId="2" r:id="R734ad9c1f74b455d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_Ratifikasi" sheetId="3" r:id="Rfd4893045e354c2f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_Change_Request" sheetId="4" r:id="Ra038528ea7eb48d7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_Kinerja" sheetId="5" r:id="R697367d433b04d69"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_Penyusunan_Kebijakan" sheetId="6" r:id="R78f1d1e7d2d04053"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_Business_Excellence" sheetId="7" r:id="R82c16b25299d43bc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_Ringkasan" sheetId="8" r:id="Rb2defee5db974015"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -716,7 +716,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6a9772622de2458c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1381f517df9647ad"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -807,7 +807,9 @@
       <x:c r="D5" s="9" t="n">
         <x:v>50</x:v>
       </x:c>
-      <x:c r="E5" s="9" t="str"/>
+      <x:c r="E5" s="9" t="str">
+        <x:v>Status sumber: Review Legal</x:v>
+      </x:c>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="9" t="str">
@@ -822,7 +824,9 @@
       <x:c r="D6" s="9" t="n">
         <x:v>50</x:v>
       </x:c>
-      <x:c r="E6" s="9" t="str"/>
+      <x:c r="E6" s="9" t="str">
+        <x:v>Status sumber: Review Legal</x:v>
+      </x:c>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="9" t="str">
@@ -837,7 +841,9 @@
       <x:c r="D7" s="9" t="n">
         <x:v>50</x:v>
       </x:c>
-      <x:c r="E7" s="9" t="str"/>
+      <x:c r="E7" s="9" t="str">
+        <x:v>Status sumber: Review Legal</x:v>
+      </x:c>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="9" t="str">
@@ -852,7 +858,9 @@
       <x:c r="D8" s="9" t="n">
         <x:v>50</x:v>
       </x:c>
-      <x:c r="E8" s="9" t="str"/>
+      <x:c r="E8" s="9" t="str">
+        <x:v>Status sumber: Review Legal</x:v>
+      </x:c>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="9" t="str">
@@ -867,7 +875,9 @@
       <x:c r="D9" s="9" t="n">
         <x:v>50</x:v>
       </x:c>
-      <x:c r="E9" s="9" t="str"/>
+      <x:c r="E9" s="9" t="str">
+        <x:v>Status sumber: Review Legal</x:v>
+      </x:c>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="9" t="str">
@@ -882,7 +892,9 @@
       <x:c r="D10" s="9" t="n">
         <x:v>50</x:v>
       </x:c>
-      <x:c r="E10" s="9" t="str"/>
+      <x:c r="E10" s="9" t="str">
+        <x:v>Status sumber: Review Legal</x:v>
+      </x:c>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="9" t="str">
@@ -897,7 +909,9 @@
       <x:c r="D11" s="9" t="n">
         <x:v>50</x:v>
       </x:c>
-      <x:c r="E11" s="9" t="str"/>
+      <x:c r="E11" s="9" t="str">
+        <x:v>Status sumber: Review Legal</x:v>
+      </x:c>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="9" t="str">
@@ -912,7 +926,9 @@
       <x:c r="D12" s="9" t="n">
         <x:v>50</x:v>
       </x:c>
-      <x:c r="E12" s="9" t="str"/>
+      <x:c r="E12" s="9" t="str">
+        <x:v>Status sumber: Review Legal</x:v>
+      </x:c>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="9" t="str">
@@ -927,7 +943,9 @@
       <x:c r="D13" s="9" t="n">
         <x:v>50</x:v>
       </x:c>
-      <x:c r="E13" s="9" t="str"/>
+      <x:c r="E13" s="9" t="str">
+        <x:v>Status sumber: Review Legal</x:v>
+      </x:c>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="9" t="str">
@@ -942,7 +960,9 @@
       <x:c r="D14" s="9" t="n">
         <x:v>50</x:v>
       </x:c>
-      <x:c r="E14" s="9" t="str"/>
+      <x:c r="E14" s="9" t="str">
+        <x:v>Status sumber: Proses Pengesahan</x:v>
+      </x:c>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="9" t="str">
@@ -957,7 +977,9 @@
       <x:c r="D15" s="9" t="n">
         <x:v>50</x:v>
       </x:c>
-      <x:c r="E15" s="9" t="str"/>
+      <x:c r="E15" s="9" t="str">
+        <x:v>Status sumber: Review Legal</x:v>
+      </x:c>
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="9" t="str">
@@ -972,7 +994,9 @@
       <x:c r="D16" s="9" t="n">
         <x:v>50</x:v>
       </x:c>
-      <x:c r="E16" s="9" t="str"/>
+      <x:c r="E16" s="9" t="str">
+        <x:v>Status sumber: Proses Pengesahan</x:v>
+      </x:c>
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="9" t="str">
@@ -987,7 +1011,9 @@
       <x:c r="D17" s="9" t="n">
         <x:v>50</x:v>
       </x:c>
-      <x:c r="E17" s="9" t="str"/>
+      <x:c r="E17" s="9" t="str">
+        <x:v>Status sumber: Proses Pengesahan</x:v>
+      </x:c>
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="9" t="str">
@@ -1017,7 +1043,9 @@
       <x:c r="D19" s="9" t="n">
         <x:v>50</x:v>
       </x:c>
-      <x:c r="E19" s="9" t="str"/>
+      <x:c r="E19" s="9" t="str">
+        <x:v>Status sumber: Proses Pengesahan</x:v>
+      </x:c>
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="9" t="str">
@@ -1032,7 +1060,9 @@
       <x:c r="D20" s="9" t="n">
         <x:v>50</x:v>
       </x:c>
-      <x:c r="E20" s="9" t="str"/>
+      <x:c r="E20" s="9" t="str">
+        <x:v>Status sumber: Proses Pengesahan</x:v>
+      </x:c>
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="9" t="str">
@@ -1047,7 +1077,9 @@
       <x:c r="D21" s="9" t="n">
         <x:v>50</x:v>
       </x:c>
-      <x:c r="E21" s="9" t="str"/>
+      <x:c r="E21" s="9" t="str">
+        <x:v>Status sumber: Proses Pengesahan</x:v>
+      </x:c>
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="9" t="str">
@@ -1062,7 +1094,9 @@
       <x:c r="D22" s="9" t="n">
         <x:v>50</x:v>
       </x:c>
-      <x:c r="E22" s="9" t="str"/>
+      <x:c r="E22" s="9" t="str">
+        <x:v>Status sumber: Proses Pengesahan</x:v>
+      </x:c>
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="9" t="str">
@@ -1077,7 +1111,9 @@
       <x:c r="D23" s="9" t="n">
         <x:v>50</x:v>
       </x:c>
-      <x:c r="E23" s="9" t="str"/>
+      <x:c r="E23" s="9" t="str">
+        <x:v>Status sumber: GRC</x:v>
+      </x:c>
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="9" t="str">
@@ -1092,7 +1128,9 @@
       <x:c r="D24" s="9" t="n">
         <x:v>50</x:v>
       </x:c>
-      <x:c r="E24" s="9" t="str"/>
+      <x:c r="E24" s="9" t="str">
+        <x:v>Status sumber: GRC</x:v>
+      </x:c>
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="9" t="str">
@@ -1257,7 +1295,9 @@
       <x:c r="D35" s="9" t="n">
         <x:v>50</x:v>
       </x:c>
-      <x:c r="E35" s="9" t="str"/>
+      <x:c r="E35" s="9" t="str">
+        <x:v>Status sumber: Proses Pengesahan</x:v>
+      </x:c>
     </x:row>
     <x:row r="36">
       <x:c r="A36" s="9" t="str">
@@ -1377,7 +1417,9 @@
       <x:c r="D43" s="9" t="n">
         <x:v>50</x:v>
       </x:c>
-      <x:c r="E43" s="9" t="str"/>
+      <x:c r="E43" s="9" t="str">
+        <x:v>Status sumber: GRC</x:v>
+      </x:c>
     </x:row>
     <x:row r="44">
       <x:c r="A44" s="9" t="str">
@@ -1467,7 +1509,9 @@
       <x:c r="D49" s="9" t="n">
         <x:v>50</x:v>
       </x:c>
-      <x:c r="E49" s="9" t="str"/>
+      <x:c r="E49" s="9" t="str">
+        <x:v>Status sumber: Proses Pengesahan</x:v>
+      </x:c>
     </x:row>
     <x:row r="50">
       <x:c r="A50" s="9" t="str">
@@ -1677,7 +1721,9 @@
       <x:c r="D63" s="9" t="n">
         <x:v>50</x:v>
       </x:c>
-      <x:c r="E63" s="9" t="str"/>
+      <x:c r="E63" s="9" t="str">
+        <x:v>Status sumber: Proses Pengesahan</x:v>
+      </x:c>
     </x:row>
     <x:row r="64">
       <x:c r="A64" s="9" t="str">
@@ -1812,7 +1858,9 @@
       <x:c r="D72" s="9" t="n">
         <x:v>50</x:v>
       </x:c>
-      <x:c r="E72" s="9" t="str"/>
+      <x:c r="E72" s="9" t="str">
+        <x:v>Status sumber: Proses Pengesahan</x:v>
+      </x:c>
     </x:row>
     <x:row r="73">
       <x:c r="A73" s="9" t="str">
@@ -1827,7 +1875,9 @@
       <x:c r="D73" s="9" t="n">
         <x:v>50</x:v>
       </x:c>
-      <x:c r="E73" s="9" t="str"/>
+      <x:c r="E73" s="9" t="str">
+        <x:v>Status sumber: Proses Pengesahan</x:v>
+      </x:c>
     </x:row>
     <x:row r="74">
       <x:c r="A74" s="9" t="str">
@@ -1887,7 +1937,9 @@
       <x:c r="D77" s="9" t="n">
         <x:v>50</x:v>
       </x:c>
-      <x:c r="E77" s="9" t="str"/>
+      <x:c r="E77" s="9" t="str">
+        <x:v>Status sumber: Proses Pengesahan</x:v>
+      </x:c>
     </x:row>
     <x:row r="78">
       <x:c r="A78" s="9" t="str">
@@ -2097,7 +2149,9 @@
       <x:c r="D91" s="9" t="n">
         <x:v>50</x:v>
       </x:c>
-      <x:c r="E91" s="9" t="str"/>
+      <x:c r="E91" s="9" t="str">
+        <x:v>Status sumber: Proses Pengesahan</x:v>
+      </x:c>
     </x:row>
     <x:row r="92">
       <x:c r="A92" s="9" t="str">
@@ -2262,7 +2316,9 @@
       <x:c r="D102" s="9" t="n">
         <x:v>50</x:v>
       </x:c>
-      <x:c r="E102" s="9" t="str"/>
+      <x:c r="E102" s="9" t="str">
+        <x:v>Status sumber: Proses Pengesahan</x:v>
+      </x:c>
     </x:row>
     <x:row r="103">
       <x:c r="A103" s="9" t="str">
@@ -2277,7 +2333,9 @@
       <x:c r="D103" s="9" t="n">
         <x:v>50</x:v>
       </x:c>
-      <x:c r="E103" s="9" t="str"/>
+      <x:c r="E103" s="9" t="str">
+        <x:v>Status sumber: Proses Pengesahan</x:v>
+      </x:c>
     </x:row>
     <x:row r="104">
       <x:c r="A104" s="9" t="str">
@@ -2292,7 +2350,9 @@
       <x:c r="D104" s="9" t="n">
         <x:v>50</x:v>
       </x:c>
-      <x:c r="E104" s="9" t="str"/>
+      <x:c r="E104" s="9" t="str">
+        <x:v>Status sumber: Proses Pengesahan</x:v>
+      </x:c>
     </x:row>
     <x:row r="105">
       <x:c r="A105" s="9" t="str">
@@ -2307,7 +2367,9 @@
       <x:c r="D105" s="9" t="n">
         <x:v>50</x:v>
       </x:c>
-      <x:c r="E105" s="9" t="str"/>
+      <x:c r="E105" s="9" t="str">
+        <x:v>Status sumber: Proses Pengesahan</x:v>
+      </x:c>
     </x:row>
     <x:row r="106">
       <x:c r="A106" s="9" t="str">
@@ -2322,7 +2384,9 @@
       <x:c r="D106" s="9" t="n">
         <x:v>50</x:v>
       </x:c>
-      <x:c r="E106" s="9" t="str"/>
+      <x:c r="E106" s="9" t="str">
+        <x:v>Status sumber: Proses Pengesahan</x:v>
+      </x:c>
     </x:row>
     <x:row r="107">
       <x:c r="A107" s="9" t="str">
@@ -2337,7 +2401,9 @@
       <x:c r="D107" s="9" t="n">
         <x:v>50</x:v>
       </x:c>
-      <x:c r="E107" s="9" t="str"/>
+      <x:c r="E107" s="9" t="str">
+        <x:v>Status sumber: Proses Pengesahan</x:v>
+      </x:c>
     </x:row>
     <x:row r="108">
       <x:c r="A108" s="9" t="str">
@@ -2352,7 +2418,9 @@
       <x:c r="D108" s="9" t="n">
         <x:v>50</x:v>
       </x:c>
-      <x:c r="E108" s="9" t="str"/>
+      <x:c r="E108" s="9" t="str">
+        <x:v>Status sumber: Proses Pengesahan</x:v>
+      </x:c>
     </x:row>
     <x:row r="109">
       <x:c r="A109" s="9" t="str">
@@ -2397,7 +2465,9 @@
       <x:c r="D111" s="9" t="n">
         <x:v>50</x:v>
       </x:c>
-      <x:c r="E111" s="9" t="str"/>
+      <x:c r="E111" s="9" t="str">
+        <x:v>Status sumber: Proses Pengesahan</x:v>
+      </x:c>
     </x:row>
     <x:row r="112">
       <x:c r="A112" s="9" t="str">
@@ -2517,7 +2587,9 @@
       <x:c r="D119" s="9" t="n">
         <x:v>50</x:v>
       </x:c>
-      <x:c r="E119" s="9" t="str"/>
+      <x:c r="E119" s="9" t="str">
+        <x:v>Status sumber: Proses Pengesahan</x:v>
+      </x:c>
     </x:row>
     <x:row r="120">
       <x:c r="A120" s="9" t="str">
@@ -2727,7 +2799,9 @@
       <x:c r="D133" s="9" t="n">
         <x:v>50</x:v>
       </x:c>
-      <x:c r="E133" s="9" t="str"/>
+      <x:c r="E133" s="9" t="str">
+        <x:v>Status sumber: Proses Pengesahan</x:v>
+      </x:c>
     </x:row>
     <x:row r="134">
       <x:c r="A134" s="9" t="str">
@@ -2857,7 +2931,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3e7410fd87ab4cd6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re4396c8e007c4120"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3051,7 +3125,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc02bf1138dad451b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rce082ba897114069"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3610,7 +3684,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6a17f4ba8dca4325"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R955a39553960440e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3715,7 +3789,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6eb8f7807c0d4a90"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd95bc6dc54b64928"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3805,7 +3879,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdaeefcabd3474a28"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3111bb607b8f4d36"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3910,7 +3984,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra8a71c537aa54c4d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbc2e674b2d1b43f1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>